<commit_message>
some what working code
</commit_message>
<xml_diff>
--- a/TIME TABLE SAMPLE DATA/INPUTS/LAB.xlsx
+++ b/TIME TABLE SAMPLE DATA/INPUTS/LAB.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rajas\OneDrive\Desktop\Timetable\TIME TABLE SAMPLE DATA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5afc8f5c19c83632/Desktop/Timetable/TIME TABLE SAMPLE DATA/INPUTS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C785179B-C7D6-42C7-9F76-C1A75874E627}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{C785179B-C7D6-42C7-9F76-C1A75874E627}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DE9B1F16-B8AC-464C-BB35-99003570C849}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BCF9C078-864F-461E-980E-EDA7976046E4}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="24">
   <si>
     <t>YEAR</t>
   </si>
@@ -106,9 +106,6 @@
   </si>
   <si>
     <t>1,2,3</t>
-  </si>
-  <si>
-    <t>GROUND</t>
   </si>
 </sst>
 </file>
@@ -486,7 +483,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{762F231F-A71F-4894-BFCC-34A32DE3DF15}">
-  <dimension ref="A1:F85"/>
+  <dimension ref="A1:F74"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="12.44140625" customWidth="1"/>
@@ -1414,222 +1411,222 @@
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B47" t="s">
         <v>10</v>
       </c>
       <c r="C47">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D47">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E47" t="s">
-        <v>11</v>
-      </c>
-      <c r="F47" t="s">
-        <v>24</v>
+        <v>17</v>
+      </c>
+      <c r="F47">
+        <v>2303</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B48" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C48">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D48">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E48" t="s">
-        <v>11</v>
-      </c>
-      <c r="F48" t="s">
-        <v>24</v>
+        <v>17</v>
+      </c>
+      <c r="F48">
+        <v>2303</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B49" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C49">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D49">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E49" t="s">
-        <v>11</v>
-      </c>
-      <c r="F49" t="s">
-        <v>24</v>
+        <v>17</v>
+      </c>
+      <c r="F49">
+        <v>2303</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B50" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="C50">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D50">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E50" t="s">
-        <v>11</v>
-      </c>
-      <c r="F50" t="s">
-        <v>24</v>
+        <v>17</v>
+      </c>
+      <c r="F50">
+        <v>2301</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B51" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="C51">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D51">
         <v>5</v>
       </c>
       <c r="E51" t="s">
-        <v>11</v>
-      </c>
-      <c r="F51" t="s">
-        <v>24</v>
+        <v>17</v>
+      </c>
+      <c r="F51">
+        <v>2301</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B52" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="C52">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D52">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E52" t="s">
-        <v>11</v>
-      </c>
-      <c r="F52" t="s">
-        <v>24</v>
+        <v>17</v>
+      </c>
+      <c r="F52">
+        <v>2301</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B53" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C53">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D53">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E53" t="s">
-        <v>11</v>
-      </c>
-      <c r="F53" t="s">
-        <v>24</v>
+        <v>17</v>
+      </c>
+      <c r="F53">
+        <v>2302</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B54" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="C54">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D54">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E54" t="s">
-        <v>11</v>
-      </c>
-      <c r="F54" t="s">
-        <v>24</v>
+        <v>17</v>
+      </c>
+      <c r="F54">
+        <v>2302</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B55" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C55">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D55">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E55" t="s">
-        <v>11</v>
-      </c>
-      <c r="F55" t="s">
-        <v>24</v>
+        <v>17</v>
+      </c>
+      <c r="F55">
+        <v>2302</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B56" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="C56">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D56">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E56" t="s">
-        <v>11</v>
-      </c>
-      <c r="F56" t="s">
-        <v>24</v>
+        <v>17</v>
+      </c>
+      <c r="F56">
+        <v>2301</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B57" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="C57">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D57">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E57" t="s">
-        <v>11</v>
-      </c>
-      <c r="F57" t="s">
-        <v>24</v>
+        <v>17</v>
+      </c>
+      <c r="F57">
+        <v>2301</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
@@ -1637,19 +1634,19 @@
         <v>3</v>
       </c>
       <c r="B58" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C58">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D58">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E58" t="s">
         <v>17</v>
       </c>
       <c r="F58">
-        <v>2303</v>
+        <v>2301</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.3">
@@ -1657,19 +1654,19 @@
         <v>3</v>
       </c>
       <c r="B59" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C59">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D59">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E59" t="s">
         <v>17</v>
       </c>
       <c r="F59">
-        <v>2303</v>
+        <v>2302</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.3">
@@ -1677,19 +1674,19 @@
         <v>3</v>
       </c>
       <c r="B60" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C60">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D60">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E60" t="s">
         <v>17</v>
       </c>
       <c r="F60">
-        <v>2303</v>
+        <v>2302</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
@@ -1697,19 +1694,19 @@
         <v>3</v>
       </c>
       <c r="B61" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="C61">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D61">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E61" t="s">
         <v>17</v>
       </c>
       <c r="F61">
-        <v>2301</v>
+        <v>2302</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
@@ -1717,19 +1714,19 @@
         <v>3</v>
       </c>
       <c r="B62" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C62">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D62">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E62" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="F62">
-        <v>2301</v>
+        <v>2302</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
@@ -1740,16 +1737,16 @@
         <v>6</v>
       </c>
       <c r="C63">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D63">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E63" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="F63">
-        <v>2301</v>
+        <v>2303</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
@@ -1760,13 +1757,13 @@
         <v>14</v>
       </c>
       <c r="C64">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D64">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E64" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="F64">
         <v>2302</v>
@@ -1777,16 +1774,16 @@
         <v>3</v>
       </c>
       <c r="B65" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C65">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D65">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E65" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="F65">
         <v>2302</v>
@@ -1797,16 +1794,16 @@
         <v>3</v>
       </c>
       <c r="B66" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C66">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D66">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E66" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="F66">
         <v>2302</v>
@@ -1817,19 +1814,19 @@
         <v>3</v>
       </c>
       <c r="B67" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="C67">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D67">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E67" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="F67">
-        <v>2301</v>
+        <v>2303</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
@@ -1837,16 +1834,16 @@
         <v>3</v>
       </c>
       <c r="B68" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C68">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D68">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E68" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="F68">
         <v>2301</v>
@@ -1857,19 +1854,19 @@
         <v>3</v>
       </c>
       <c r="B69" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="C69">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D69">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E69" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="F69">
-        <v>2301</v>
+        <v>2303</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
@@ -1877,19 +1874,19 @@
         <v>3</v>
       </c>
       <c r="B70" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="C70">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D70">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E70" t="s">
         <v>17</v>
       </c>
       <c r="F70">
-        <v>2302</v>
+        <v>2303</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.3">
@@ -1897,19 +1894,19 @@
         <v>3</v>
       </c>
       <c r="B71" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="C71">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D71">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E71" t="s">
         <v>17</v>
       </c>
       <c r="F71">
-        <v>2302</v>
+        <v>2303</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.3">
@@ -1917,19 +1914,19 @@
         <v>3</v>
       </c>
       <c r="B72" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C72">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D72">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E72" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="F72">
-        <v>2302</v>
+        <v>2301</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.3">
@@ -1937,19 +1934,19 @@
         <v>3</v>
       </c>
       <c r="B73" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C73">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D73">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E73" t="s">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="F73">
-        <v>2302</v>
+        <v>2301</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.3">
@@ -1957,238 +1954,18 @@
         <v>3</v>
       </c>
       <c r="B74" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="C74">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D74">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E74" t="s">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="F74">
-        <v>2303</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A75">
-        <v>3</v>
-      </c>
-      <c r="B75" t="s">
-        <v>14</v>
-      </c>
-      <c r="C75">
-        <v>20</v>
-      </c>
-      <c r="D75">
-        <v>2</v>
-      </c>
-      <c r="E75" t="s">
-        <v>7</v>
-      </c>
-      <c r="F75">
-        <v>2302</v>
-      </c>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A76">
-        <v>3</v>
-      </c>
-      <c r="B76" t="s">
-        <v>13</v>
-      </c>
-      <c r="C76">
-        <v>20</v>
-      </c>
-      <c r="D76">
-        <v>5</v>
-      </c>
-      <c r="E76" t="s">
-        <v>9</v>
-      </c>
-      <c r="F76">
-        <v>2302</v>
-      </c>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A77">
-        <v>3</v>
-      </c>
-      <c r="B77" t="s">
-        <v>12</v>
-      </c>
-      <c r="C77">
-        <v>20</v>
-      </c>
-      <c r="D77">
-        <v>4</v>
-      </c>
-      <c r="E77" t="s">
-        <v>7</v>
-      </c>
-      <c r="F77">
-        <v>2302</v>
-      </c>
-    </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A78">
-        <v>3</v>
-      </c>
-      <c r="B78" t="s">
-        <v>19</v>
-      </c>
-      <c r="C78">
-        <v>20</v>
-      </c>
-      <c r="D78">
-        <v>2</v>
-      </c>
-      <c r="E78" t="s">
-        <v>7</v>
-      </c>
-      <c r="F78">
-        <v>2303</v>
-      </c>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A79">
-        <v>3</v>
-      </c>
-      <c r="B79" t="s">
-        <v>15</v>
-      </c>
-      <c r="C79">
-        <v>20</v>
-      </c>
-      <c r="D79">
-        <v>4</v>
-      </c>
-      <c r="E79" t="s">
-        <v>9</v>
-      </c>
-      <c r="F79">
-        <v>2301</v>
-      </c>
-    </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A80">
-        <v>3</v>
-      </c>
-      <c r="B80" t="s">
-        <v>19</v>
-      </c>
-      <c r="C80">
-        <v>17</v>
-      </c>
-      <c r="D80">
-        <v>4</v>
-      </c>
-      <c r="E80" t="s">
-        <v>23</v>
-      </c>
-      <c r="F80">
-        <v>2303</v>
-      </c>
-    </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A81">
-        <v>3</v>
-      </c>
-      <c r="B81" t="s">
-        <v>19</v>
-      </c>
-      <c r="C81">
-        <v>18</v>
-      </c>
-      <c r="D81">
-        <v>5</v>
-      </c>
-      <c r="E81" t="s">
-        <v>17</v>
-      </c>
-      <c r="F81">
-        <v>2303</v>
-      </c>
-    </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A82">
-        <v>3</v>
-      </c>
-      <c r="B82" t="s">
-        <v>19</v>
-      </c>
-      <c r="C82">
-        <v>19</v>
-      </c>
-      <c r="D82">
-        <v>6</v>
-      </c>
-      <c r="E82" t="s">
-        <v>17</v>
-      </c>
-      <c r="F82">
-        <v>2303</v>
-      </c>
-    </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A83">
-        <v>3</v>
-      </c>
-      <c r="B83" t="s">
-        <v>15</v>
-      </c>
-      <c r="C83">
-        <v>17</v>
-      </c>
-      <c r="D83">
-        <v>1</v>
-      </c>
-      <c r="E83" t="s">
-        <v>23</v>
-      </c>
-      <c r="F83">
-        <v>2301</v>
-      </c>
-    </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A84">
-        <v>3</v>
-      </c>
-      <c r="B84" t="s">
-        <v>15</v>
-      </c>
-      <c r="C84">
-        <v>18</v>
-      </c>
-      <c r="D84">
-        <v>2</v>
-      </c>
-      <c r="E84" t="s">
-        <v>22</v>
-      </c>
-      <c r="F84">
-        <v>2301</v>
-      </c>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A85">
-        <v>3</v>
-      </c>
-      <c r="B85" t="s">
-        <v>15</v>
-      </c>
-      <c r="C85">
-        <v>19</v>
-      </c>
-      <c r="D85">
-        <v>3</v>
-      </c>
-      <c r="E85" t="s">
-        <v>23</v>
-      </c>
-      <c r="F85">
         <v>2301</v>
       </c>
     </row>

</xml_diff>